<commit_message>
Update CW data 2026-10-30
</commit_message>
<xml_diff>
--- a/docs/downloads/ThongTinChungQuyen_latest.xlsx
+++ b/docs/downloads/ThongTinChungQuyen_latest.xlsx
@@ -5705,7 +5705,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>11,000,000</t>
+          <t>16,000,000</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -10409,7 +10409,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>11,000,000</t>
+          <t>16,000,000</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>15,000,000</t>
+          <t>20,000,000</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -12215,7 +12215,7 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>11,000,000</t>
+          <t>16,000,000</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>11,000,000</t>
+          <t>16,000,000</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">

</xml_diff>